<commit_message>
Alles für Mainscreen Prototyp
</commit_message>
<xml_diff>
--- a/Organisation/Charaktere und Eigenschaften.xlsx
+++ b/Organisation/Charaktere und Eigenschaften.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katharina\Documents\GitHub\WiesnKrisn\Organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C079AF-BA2A-4FC7-9F37-A0781DD5DA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3609852B-2A9E-4121-A8C3-5073336D934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DA5F6F0B-22DD-4C3C-AF2B-292FE63D117F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DA5F6F0B-22DD-4C3C-AF2B-292FE63D117F}"/>
   </bookViews>
   <sheets>
     <sheet name="Charaktere" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="112">
   <si>
     <t>Aperoli 2 (Ali)</t>
   </si>
@@ -366,6 +366,18 @@
   </si>
   <si>
     <t>Schwirigkeitsgrad</t>
+  </si>
+  <si>
+    <t>Pause</t>
+  </si>
+  <si>
+    <t>fortsetzen</t>
+  </si>
+  <si>
+    <t>hauptmenü</t>
+  </si>
+  <si>
+    <t>einstellungen</t>
   </si>
 </sst>
 </file>
@@ -716,7 +728,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
@@ -738,27 +750,20 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1093,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3195D32-BEA3-45FA-824D-F95B39CF5191}">
-  <dimension ref="A1:O64"/>
+  <dimension ref="B1:L64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.28515625" customWidth="1"/>
@@ -1103,8 +1108,8 @@
     <col min="14" max="14" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="15" t="s">
         <v>5</v>
       </c>
@@ -1136,7 +1141,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="18" t="s">
         <v>89</v>
       </c>
@@ -1171,7 +1176,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
         <v>90</v>
       </c>
@@ -1206,7 +1211,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="19" t="s">
         <v>93</v>
       </c>
@@ -1241,7 +1246,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="19" t="s">
         <v>0</v>
       </c>
@@ -1276,7 +1281,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="19" t="s">
         <v>85</v>
       </c>
@@ -1311,7 +1316,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>2</v>
       </c>
@@ -1346,7 +1351,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="19" t="s">
         <v>87</v>
       </c>
@@ -1381,7 +1386,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="19" t="s">
         <v>91</v>
       </c>
@@ -1416,7 +1421,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="19" t="s">
         <v>92</v>
       </c>
@@ -1451,7 +1456,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="20" t="s">
         <v>64</v>
       </c>
@@ -1486,44 +1491,13 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="21"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="21"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="21"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="21"/>
-      <c r="B14" s="28" t="s">
+    <row r="13" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="21"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="21"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="18" t="s">
         <v>80</v>
       </c>
@@ -1554,93 +1528,81 @@
       <c r="K15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="29" t="s">
+      <c r="L15" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="21"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="21"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="21"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="23" t="s">
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="27"/>
+      <c r="C16" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="F16" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="23" t="s">
+      <c r="H16" t="s">
         <v>34</v>
       </c>
-      <c r="I16" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="J16" s="23" t="s">
+      <c r="I16" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16" t="s">
         <v>37</v>
       </c>
-      <c r="K16" s="23" t="s">
+      <c r="K16" t="s">
         <v>39</v>
       </c>
-      <c r="L16" s="31" t="s">
+      <c r="L16" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="M16" s="21"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="21"/>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="21"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="33" t="s">
+    </row>
+    <row r="17" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="29"/>
+      <c r="C17" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="33" t="s">
+      <c r="D17" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="33" t="s">
+      <c r="E17" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="33" t="s">
+      <c r="F17" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="G17" s="33" t="s">
+      <c r="G17" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="33" t="s">
+      <c r="H17" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="33" t="s">
+      <c r="I17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="J17" s="33" t="s">
+      <c r="J17" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="K17" s="33" t="s">
+      <c r="K17" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="L17" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="M17" s="21"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="21"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="21"/>
+      <c r="L17" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="32" t="s">
         <v>24</v>
       </c>
       <c r="D18" s="14" t="s">
@@ -1667,86 +1629,78 @@
       <c r="K18" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="L18" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="M18" s="21"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="21"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="21"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="23" t="s">
+      <c r="L18" s="33" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="27"/>
+      <c r="C19" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" t="s">
         <v>27</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="23" t="s">
+      <c r="G19" t="s">
         <v>33</v>
       </c>
-      <c r="H19" s="23" t="s">
+      <c r="H19" t="s">
         <v>34</v>
       </c>
-      <c r="I19" s="23" t="s">
+      <c r="I19" t="s">
         <v>21</v>
       </c>
-      <c r="J19" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="K19" s="23" t="s">
+      <c r="J19" t="s">
+        <v>22</v>
+      </c>
+      <c r="K19" t="s">
         <v>40</v>
       </c>
-      <c r="L19" s="31" t="s">
+      <c r="L19" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="M19" s="21"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="21"/>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="37"/>
-      <c r="C20" s="33" t="s">
+    </row>
+    <row r="20" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="29"/>
+      <c r="C20" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="33" t="s">
+      <c r="D20" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="38" t="s">
+      <c r="E20" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F20" s="38" t="s">
+      <c r="F20" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G20" s="38" t="s">
+      <c r="G20" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="38" t="s">
+      <c r="H20" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="I20" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J20" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="K20" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="L20" s="39" t="s">
+      <c r="I20" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J20" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="K20" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="L20" s="31" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="21"/>
-      <c r="B21" s="28" t="s">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="25" t="s">
         <v>82</v>
       </c>
       <c r="C21" s="4" t="s">
@@ -1779,86 +1733,74 @@
       <c r="L21" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="M21" s="21"/>
-      <c r="N21" s="23"/>
-      <c r="O21" s="21"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="21"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="23" t="s">
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="27"/>
+      <c r="C22" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="23" t="s">
+      <c r="D22" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" t="s">
         <v>17</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="F22" t="s">
         <v>31</v>
       </c>
-      <c r="G22" s="23" t="s">
+      <c r="G22" t="s">
         <v>32</v>
       </c>
-      <c r="H22" s="23" t="s">
+      <c r="H22" t="s">
         <v>35</v>
       </c>
-      <c r="I22" s="23" t="s">
+      <c r="I22" t="s">
         <v>21</v>
       </c>
-      <c r="J22" s="23" t="s">
+      <c r="J22" t="s">
         <v>37</v>
       </c>
-      <c r="K22" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="L22" s="31" t="s">
+      <c r="K22" t="s">
+        <v>22</v>
+      </c>
+      <c r="L22" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="M22" s="21"/>
-      <c r="N22" s="23"/>
-      <c r="O22" s="21"/>
-    </row>
-    <row r="23" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="21"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="33" t="s">
+    </row>
+    <row r="23" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="29"/>
+      <c r="C23" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="33" t="s">
+      <c r="E23" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="33" t="s">
+      <c r="F23" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="G23" s="33" t="s">
+      <c r="G23" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="33" t="s">
+      <c r="H23" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="33" t="s">
+      <c r="I23" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="J23" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="K23" s="33" t="s">
+      <c r="J23" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="K23" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="L23" s="34" t="s">
+      <c r="L23" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="M23" s="21"/>
-      <c r="N23" s="23"/>
-      <c r="O23" s="21"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="21"/>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
         <v>83</v>
       </c>
@@ -1892,86 +1834,74 @@
       <c r="L24" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M24" s="21"/>
-      <c r="N24" s="23"/>
-      <c r="O24" s="21"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="23" t="s">
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="27"/>
+      <c r="C25" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="F25" t="s">
         <v>30</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="G25" t="s">
         <v>33</v>
       </c>
-      <c r="H25" s="23" t="s">
+      <c r="H25" t="s">
         <v>35</v>
       </c>
-      <c r="I25" s="23" t="s">
+      <c r="I25" t="s">
         <v>21</v>
       </c>
-      <c r="J25" s="23" t="s">
+      <c r="J25" t="s">
         <v>38</v>
       </c>
-      <c r="K25" s="23" t="s">
+      <c r="K25" t="s">
         <v>39</v>
       </c>
-      <c r="L25" s="31" t="s">
+      <c r="L25" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="M25" s="21"/>
-      <c r="N25" s="23"/>
-      <c r="O25" s="21"/>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="21"/>
-      <c r="B26" s="37"/>
-      <c r="C26" s="33" t="s">
+    </row>
+    <row r="26" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="29"/>
+      <c r="C26" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D26" s="33" t="s">
+      <c r="D26" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E26" s="33" t="s">
+      <c r="E26" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="33" t="s">
+      <c r="F26" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G26" s="33" t="s">
+      <c r="G26" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="H26" s="33" t="s">
+      <c r="H26" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="I26" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="33" t="s">
+      <c r="I26" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="K26" s="33" t="s">
+      <c r="K26" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="L26" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="M26" s="21"/>
-      <c r="N26" s="23"/>
-      <c r="O26" s="21"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="21"/>
+      <c r="L26" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="18" t="s">
         <v>85</v>
       </c>
@@ -2005,86 +1935,74 @@
       <c r="L27" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="M27" s="21"/>
-      <c r="N27" s="23"/>
-      <c r="O27" s="21"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="21"/>
-      <c r="B28" s="40"/>
-      <c r="C28" s="23" t="s">
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="34"/>
+      <c r="C28" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" t="s">
         <v>96</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="23" t="s">
+      <c r="F28" t="s">
         <v>18</v>
       </c>
-      <c r="G28" s="23" t="s">
+      <c r="G28" t="s">
         <v>32</v>
       </c>
-      <c r="H28" s="23" t="s">
+      <c r="H28" t="s">
         <v>35</v>
       </c>
-      <c r="I28" s="23" t="s">
+      <c r="I28" t="s">
         <v>21</v>
       </c>
-      <c r="J28" s="23" t="s">
+      <c r="J28" t="s">
         <v>37</v>
       </c>
-      <c r="K28" s="23" t="s">
+      <c r="K28" t="s">
         <v>95</v>
       </c>
-      <c r="L28" s="31" t="s">
+      <c r="L28" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="M28" s="21"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="21"/>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="21"/>
-      <c r="B29" s="27"/>
-      <c r="C29" s="33" t="s">
+    </row>
+    <row r="29" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="24"/>
+      <c r="C29" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="E29" s="33" t="s">
+      <c r="E29" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="F29" s="33" t="s">
+      <c r="F29" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="G29" s="33" t="s">
+      <c r="G29" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="H29" s="33" t="s">
+      <c r="H29" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="I29" s="33" t="s">
+      <c r="I29" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="J29" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="K29" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="L29" s="34" t="s">
+      <c r="J29" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="K29" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="L29" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="M29" s="21"/>
-      <c r="N29" s="23"/>
-      <c r="O29" s="21"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="21"/>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="18" t="s">
         <v>84</v>
       </c>
@@ -2118,86 +2036,74 @@
       <c r="L30" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="M30" s="21"/>
-      <c r="N30" s="23"/>
-      <c r="O30" s="21"/>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="21"/>
-      <c r="B31" s="30"/>
-      <c r="C31" s="23" t="s">
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="27"/>
+      <c r="C31" t="s">
         <v>24</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" t="s">
         <v>96</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="E31" t="s">
         <v>34</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="F31" t="s">
         <v>30</v>
       </c>
-      <c r="G31" s="23" t="s">
+      <c r="G31" t="s">
         <v>32</v>
       </c>
-      <c r="H31" s="23" t="s">
+      <c r="H31" t="s">
         <v>34</v>
       </c>
-      <c r="I31" s="23" t="s">
+      <c r="I31" t="s">
         <v>36</v>
       </c>
-      <c r="J31" s="23" t="s">
+      <c r="J31" t="s">
         <v>38</v>
       </c>
-      <c r="K31" s="23" t="s">
+      <c r="K31" t="s">
         <v>39</v>
       </c>
-      <c r="L31" s="31" t="s">
+      <c r="L31" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="M31" s="21"/>
-      <c r="N31" s="23"/>
-      <c r="O31" s="21"/>
-    </row>
-    <row r="32" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="21"/>
-      <c r="B32" s="37"/>
-      <c r="C32" s="33" t="s">
+    </row>
+    <row r="32" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="29"/>
+      <c r="C32" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="E32" s="33" t="s">
+      <c r="E32" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="F32" s="33" t="s">
+      <c r="F32" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="G32" s="33" t="s">
+      <c r="G32" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="H32" s="33" t="s">
+      <c r="H32" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="I32" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="J32" s="33" t="s">
+      <c r="I32" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J32" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="K32" s="33" t="s">
+      <c r="K32" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="L32" s="34" t="s">
+      <c r="L32" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="M32" s="21"/>
-      <c r="N32" s="23"/>
-      <c r="O32" s="21"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="21"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="18" t="s">
         <v>86</v>
       </c>
@@ -2231,86 +2137,74 @@
       <c r="L33" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="M33" s="21"/>
-      <c r="N33" s="23"/>
-      <c r="O33" s="21"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="21"/>
-      <c r="B34" s="40"/>
-      <c r="C34" s="23" t="s">
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B34" s="34"/>
+      <c r="C34" t="s">
         <v>15</v>
       </c>
-      <c r="D34" s="23" t="s">
+      <c r="D34" t="s">
         <v>16</v>
       </c>
-      <c r="E34" s="23" t="s">
+      <c r="E34" t="s">
         <v>35</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="F34" t="s">
         <v>30</v>
       </c>
-      <c r="G34" s="23" t="s">
+      <c r="G34" t="s">
         <v>33</v>
       </c>
-      <c r="H34" s="23" t="s">
+      <c r="H34" t="s">
         <v>20</v>
       </c>
-      <c r="I34" s="23" t="s">
+      <c r="I34" t="s">
         <v>21</v>
       </c>
-      <c r="J34" s="23" t="s">
+      <c r="J34" t="s">
         <v>38</v>
       </c>
-      <c r="K34" s="23" t="s">
+      <c r="K34" t="s">
         <v>99</v>
       </c>
-      <c r="L34" s="31" t="s">
+      <c r="L34" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="M34" s="21"/>
-      <c r="N34" s="23"/>
-      <c r="O34" s="21"/>
-    </row>
-    <row r="35" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="21"/>
-      <c r="B35" s="27"/>
-      <c r="C35" s="33" t="s">
+    </row>
+    <row r="35" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="24"/>
+      <c r="C35" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="D35" s="33" t="s">
+      <c r="D35" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E35" s="33" t="s">
+      <c r="E35" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="F35" s="33" t="s">
+      <c r="F35" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G35" s="33" t="s">
+      <c r="G35" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="H35" s="33" t="s">
+      <c r="H35" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="I35" s="33" t="s">
+      <c r="I35" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="J35" s="33" t="s">
+      <c r="J35" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="K35" s="33" t="s">
+      <c r="K35" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="L35" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="M35" s="21"/>
-      <c r="N35" s="23"/>
-      <c r="O35" s="21"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="21"/>
+      <c r="L35" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="18" t="s">
         <v>47</v>
       </c>
@@ -2344,86 +2238,74 @@
       <c r="L36" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M36" s="21"/>
-      <c r="N36" s="23"/>
-      <c r="O36" s="21"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="21"/>
-      <c r="B37" s="40"/>
-      <c r="C37" s="23" t="s">
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B37" s="34"/>
+      <c r="C37" t="s">
         <v>100</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="D37" t="s">
         <v>16</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" t="s">
         <v>38</v>
       </c>
-      <c r="F37" s="23" t="s">
+      <c r="F37" t="s">
         <v>101</v>
       </c>
-      <c r="G37" s="23" t="s">
+      <c r="G37" t="s">
         <v>32</v>
       </c>
-      <c r="H37" s="23" t="s">
+      <c r="H37" t="s">
         <v>34</v>
       </c>
-      <c r="I37" s="23" t="s">
+      <c r="I37" t="s">
         <v>36</v>
       </c>
-      <c r="J37" s="23" t="s">
+      <c r="J37" t="s">
         <v>37</v>
       </c>
-      <c r="K37" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="L37" s="31" t="s">
+      <c r="K37" t="s">
+        <v>22</v>
+      </c>
+      <c r="L37" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="M37" s="21"/>
-      <c r="N37" s="23"/>
-      <c r="O37" s="21"/>
-    </row>
-    <row r="38" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="21"/>
-      <c r="B38" s="27"/>
-      <c r="C38" s="33" t="s">
+    </row>
+    <row r="38" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="24"/>
+      <c r="C38" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D38" s="33" t="s">
+      <c r="D38" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E38" s="33" t="s">
+      <c r="E38" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="F38" s="33" t="s">
+      <c r="F38" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="G38" s="33" t="s">
+      <c r="G38" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="H38" s="33" t="s">
+      <c r="H38" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="I38" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="J38" s="33" t="s">
+      <c r="I38" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="K38" s="33" t="s">
+      <c r="K38" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="L38" s="34" t="s">
+      <c r="L38" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="M38" s="21"/>
-      <c r="N38" s="23"/>
-      <c r="O38" s="21"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="21"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="18" t="s">
         <v>48</v>
       </c>
@@ -2457,87 +2339,75 @@
       <c r="L39" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="M39" s="21"/>
-      <c r="N39" s="23"/>
-      <c r="O39" s="21"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="21"/>
-      <c r="B40" s="26"/>
-      <c r="C40" s="23" t="s">
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40" s="23"/>
+      <c r="C40" t="s">
         <v>15</v>
       </c>
-      <c r="D40" s="23" t="s">
+      <c r="D40" t="s">
         <v>27</v>
       </c>
-      <c r="E40" s="23" t="s">
+      <c r="E40" t="s">
         <v>34</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" t="s">
         <v>31</v>
       </c>
-      <c r="G40" s="23" t="s">
+      <c r="G40" t="s">
         <v>32</v>
       </c>
-      <c r="H40" s="23" t="s">
+      <c r="H40" t="s">
         <v>34</v>
       </c>
-      <c r="I40" s="23" t="s">
+      <c r="I40" t="s">
         <v>36</v>
       </c>
-      <c r="J40" s="23" t="s">
+      <c r="J40" t="s">
         <v>37</v>
       </c>
-      <c r="K40" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="L40" s="31" t="s">
+      <c r="K40" t="s">
+        <v>22</v>
+      </c>
+      <c r="L40" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="M40" s="21"/>
-      <c r="N40" s="23"/>
-      <c r="O40" s="21"/>
-    </row>
-    <row r="41" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="21"/>
-      <c r="B41" s="27"/>
-      <c r="C41" s="33" t="s">
+    </row>
+    <row r="41" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="24"/>
+      <c r="C41" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E41" s="33" t="s">
+      <c r="E41" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="F41" s="33" t="s">
+      <c r="F41" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G41" s="33" t="s">
+      <c r="G41" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="H41" s="33" t="s">
+      <c r="H41" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="I41" s="33" t="s">
+      <c r="I41" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="J41" s="33" t="s">
+      <c r="J41" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="K41" s="33" t="s">
+      <c r="K41" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="L41" s="34" t="s">
+      <c r="L41" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="M41" s="21"/>
-      <c r="N41" s="23"/>
-      <c r="O41" s="21"/>
-    </row>
-    <row r="42" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="21"/>
-      <c r="B42" s="22" t="s">
+    </row>
+    <row r="42" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="21" t="s">
         <v>4</v>
       </c>
       <c r="C42" s="2" t="s">
@@ -2570,92 +2440,81 @@
       <c r="L42" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M42" s="21"/>
-      <c r="N42" s="23"/>
-      <c r="O42" s="21"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="21"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="23" t="s">
+    </row>
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B43" s="27"/>
+      <c r="C43" t="s">
         <v>24</v>
       </c>
-      <c r="D43" s="23" t="s">
+      <c r="D43" t="s">
         <v>98</v>
       </c>
-      <c r="E43" s="23" t="s">
+      <c r="E43" t="s">
         <v>38</v>
       </c>
-      <c r="F43" s="23" t="s">
+      <c r="F43" t="s">
         <v>102</v>
       </c>
-      <c r="G43" s="23" t="s">
+      <c r="G43" t="s">
         <v>32</v>
       </c>
-      <c r="H43" s="23" t="s">
+      <c r="H43" t="s">
         <v>34</v>
       </c>
-      <c r="I43" s="23" t="s">
+      <c r="I43" t="s">
         <v>21</v>
       </c>
-      <c r="J43" s="23" t="s">
+      <c r="J43" t="s">
         <v>38</v>
       </c>
-      <c r="K43" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="L43" s="31" t="s">
+      <c r="K43" t="s">
+        <v>22</v>
+      </c>
+      <c r="L43" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="M43" s="21"/>
-      <c r="N43" s="23"/>
-      <c r="O43" s="21"/>
-    </row>
-    <row r="44" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="21"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="33" t="s">
+    </row>
+    <row r="44" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="29"/>
+      <c r="C44" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D44" s="33" t="s">
+      <c r="D44" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="E44" s="33" t="s">
+      <c r="E44" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="F44" s="33" t="s">
+      <c r="F44" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G44" s="33" t="s">
+      <c r="G44" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="H44" s="33" t="s">
+      <c r="H44" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="I44" s="33" t="s">
+      <c r="I44" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="J44" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="K44" s="33" t="s">
+      <c r="J44" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="K44" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="L44" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="M44" s="21"/>
-      <c r="N44" s="23"/>
-      <c r="O44" s="21"/>
-    </row>
-    <row r="46" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="22" t="s">
+      <c r="L44" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="21" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B48" s="21" t="s">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2706,27 +2565,27 @@
     </row>
     <row r="59" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="60" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="22" t="s">
+      <c r="B60" s="21" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B61" s="21" t="s">
+      <c r="B61" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="62" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B62" s="23" t="s">
+      <c r="B62" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B63" s="23" t="s">
+      <c r="B63" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B64" s="23" t="s">
+      <c r="B64" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2737,7 +2596,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D786EEF-5D36-4264-943C-3E4EA6797156}">
-  <dimension ref="B1:J14"/>
+  <dimension ref="B1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.140625" customWidth="1"/>
@@ -2750,13 +2609,13 @@
   <sheetData>
     <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="22" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="5" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="22" t="s">
         <v>54</v>
       </c>
       <c r="C6" t="s">
@@ -2786,15 +2645,12 @@
     </row>
     <row r="9" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="10" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="22" t="s">
         <v>55</v>
       </c>
       <c r="C10" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -2803,7 +2659,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{998BF4DC-EA81-4A48-BF48-12E23976DBDD}">
-  <dimension ref="B1:F12"/>
+  <dimension ref="B1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" customWidth="1"/>
@@ -2813,7 +2669,7 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="22" t="s">
         <v>68</v>
       </c>
       <c r="C2" t="s">
@@ -2831,7 +2687,7 @@
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="22" t="s">
         <v>69</v>
       </c>
       <c r="C4" t="s">
@@ -2849,7 +2705,7 @@
     </row>
     <row r="5" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="22" t="s">
         <v>70</v>
       </c>
       <c r="C6" t="s">
@@ -2861,7 +2717,7 @@
     </row>
     <row r="7" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="22" t="s">
         <v>71</v>
       </c>
       <c r="C8" t="s">
@@ -2870,13 +2726,13 @@
     </row>
     <row r="9" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="22" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="22" t="s">
         <v>103</v>
       </c>
       <c r="C12" t="s">
@@ -2890,6 +2746,21 @@
       </c>
       <c r="F12" t="s">
         <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" t="s">
+        <v>109</v>
+      </c>
+      <c r="D14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2899,55 +2770,52 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E7BF28-E4F3-41A1-A826-E8C52BECF59F}">
-  <dimension ref="B1:D13"/>
+  <dimension ref="B1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="18" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="19" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="19" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="19" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="19" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="20" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D13" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>